<commit_message>
updated to add new Eagleman script
</commit_message>
<xml_diff>
--- a/Heffner_Masterton_1975/Heffner_Masterton_1975_TableI_snapshot.xlsx
+++ b/Heffner_Masterton_1975/Heffner_Masterton_1975_TableI_snapshot.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo M1 Trait Data/Heffner_Masterton_1975/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo-M1-Trait-Data/Heffner_Masterton_1975/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{9CAD6EE9-C33D-064D-855C-6CB95E315522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8861666E-C060-154B-A41C-A14C7BF6C899}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{9CAD6EE9-C33D-064D-855C-6CB95E315522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAF15C6C-7439-0244-BA44-FD45BCAE2751}"/>
   <bookViews>
-    <workbookView xWindow="50880" yWindow="-5960" windowWidth="30340" windowHeight="20420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35200" yWindow="-5860" windowWidth="50560" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Heffner-1975-Variation in form " sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="220">
   <si>
     <t>Table I. Animals and anatomical data on which all correlations are based</t>
   </si>
@@ -506,9 +506,6 @@
     <t>Rock hyrax</t>
   </si>
   <si>
-    <t>J7</t>
-  </si>
-  <si>
     <t>Pygmy shrew</t>
   </si>
   <si>
@@ -570,9 +567,6 @@
     <t>Sheep (domestic)</t>
   </si>
   <si>
-    <t>CJ</t>
-  </si>
-  <si>
     <t>CAMPBELL et al., 1966</t>
   </si>
   <si>
@@ -685,6 +679,9 @@
   </si>
   <si>
     <t xml:space="preserve">Lagothrix lagotricha </t>
+  </si>
+  <si>
+    <t>C1</t>
   </si>
 </sst>
 </file>
@@ -1304,9 +1301,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1344,7 +1341,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1450,7 +1447,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1592,7 +1589,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1880,7 +1877,7 @@
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="23" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -1936,7 +1933,7 @@
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -1978,7 +1975,7 @@
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B28" s="4" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="K28" s="10" t="s">
         <v>39</v>
@@ -2078,7 +2075,7 @@
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B36" s="4" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H36" s="10" t="s">
         <v>58</v>
@@ -2091,6 +2088,9 @@
       <c r="A37" t="s">
         <v>32</v>
       </c>
+      <c r="C37">
+        <v>1</v>
+      </c>
       <c r="D37">
         <v>570</v>
       </c>
@@ -2113,7 +2113,7 @@
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="43" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -2426,7 +2426,7 @@
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="61" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -2733,7 +2733,7 @@
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="79" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -2803,7 +2803,7 @@
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B82" s="4" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="M82" s="10" t="s">
         <v>95</v>
@@ -2811,7 +2811,7 @@
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C83">
         <v>2</v>
@@ -2825,7 +2825,7 @@
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B84" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="K84" s="10" t="s">
         <v>96</v>
@@ -2906,7 +2906,7 @@
         <v>92</v>
       </c>
       <c r="M90" s="10" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.2">
@@ -2937,7 +2937,7 @@
         <v>93</v>
       </c>
       <c r="F92" s="10" t="s">
-        <v>104</v>
+        <v>57</v>
       </c>
       <c r="H92" s="10" t="s">
         <v>14</v>
@@ -2981,7 +2981,7 @@
     </row>
     <row r="98" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A98" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="99" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -3304,7 +3304,7 @@
     </row>
     <row r="118" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A118" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="119" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -3380,7 +3380,7 @@
     </row>
     <row r="122" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B122" s="4" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="M122" s="10" t="s">
         <v>64</v>
@@ -3610,7 +3610,7 @@
     </row>
     <row r="136" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A136" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="137" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -3832,6 +3832,9 @@
       <c r="A147" s="4" t="s">
         <v>143</v>
       </c>
+      <c r="C147">
+        <v>1</v>
+      </c>
       <c r="D147">
         <v>18</v>
       </c>
@@ -3878,7 +3881,7 @@
       </c>
       <c r="K149"/>
       <c r="L149" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="M149"/>
       <c r="N149">
@@ -3930,7 +3933,7 @@
     </row>
     <row r="154" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A154" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="155" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -3986,7 +3989,7 @@
     </row>
     <row r="157" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C157" s="10">
         <v>2</v>
@@ -4008,7 +4011,7 @@
     </row>
     <row r="158" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B158" s="4" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C158" s="10"/>
       <c r="D158" s="10"/>
@@ -4050,23 +4053,23 @@
     </row>
     <row r="160" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B160" s="4" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C160" s="10"/>
       <c r="D160" s="10"/>
       <c r="G160" s="10"/>
       <c r="H160"/>
       <c r="K160" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="M160" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="O160" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Q160" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="161" spans="1:17" x14ac:dyDescent="0.2">
@@ -4100,7 +4103,7 @@
     </row>
     <row r="162" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="B162" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C162" s="10"/>
       <c r="D162" s="10"/>
@@ -4128,7 +4131,7 @@
         <v>3</v>
       </c>
       <c r="D163" s="10">
-        <v>0.12</v>
+        <v>12</v>
       </c>
       <c r="G163" s="10"/>
       <c r="H163"/>
@@ -4151,16 +4154,16 @@
       <c r="G164" s="10"/>
       <c r="H164"/>
       <c r="M164" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="O164" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="Q164"/>
     </row>
     <row r="165" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C165" s="10">
         <v>3</v>
@@ -4196,22 +4199,22 @@
       <c r="C166" s="10"/>
       <c r="D166" s="10"/>
       <c r="F166" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H166" s="3" t="s">
         <v>115</v>
       </c>
       <c r="K166" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="M166" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="M166" s="1" t="s">
-        <v>170</v>
-      </c>
       <c r="O166" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Q166" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="167" spans="1:17" x14ac:dyDescent="0.2">
@@ -4221,8 +4224,8 @@
       <c r="C167" s="10">
         <v>2</v>
       </c>
-      <c r="D167" s="10" t="s">
-        <v>161</v>
+      <c r="D167" s="10">
+        <v>17</v>
       </c>
       <c r="G167" s="10">
         <v>9</v>
@@ -4243,23 +4246,23 @@
     </row>
     <row r="168" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B168" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C168" s="10"/>
       <c r="D168" s="10"/>
       <c r="G168" s="10"/>
       <c r="H168" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K168" t="s">
         <v>14</v>
       </c>
       <c r="M168" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O168"/>
       <c r="Q168" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="169" spans="1:17" x14ac:dyDescent="0.2">
@@ -4283,7 +4286,7 @@
     </row>
     <row r="172" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A172" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="173" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -4339,7 +4342,7 @@
     </row>
     <row r="175" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C175">
         <v>1</v>
@@ -4366,14 +4369,14 @@
     </row>
     <row r="176" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B176" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F176" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="G176" s="10"/>
       <c r="H176" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="J176" s="10"/>
       <c r="K176" t="s">
@@ -4387,7 +4390,7 @@
     </row>
     <row r="177" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C177">
         <v>1</v>
@@ -4408,7 +4411,7 @@
         <v>1.42</v>
       </c>
       <c r="L177" t="s">
-        <v>182</v>
+        <v>219</v>
       </c>
       <c r="N177" s="10"/>
       <c r="O177"/>
@@ -4418,7 +4421,7 @@
     </row>
     <row r="178" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B178" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F178" t="s">
         <v>57</v>
@@ -4432,16 +4435,16 @@
         <v>57</v>
       </c>
       <c r="M178" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="O178"/>
       <c r="Q178" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="179" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C179" s="10">
         <v>5</v>
@@ -4472,7 +4475,7 @@
     </row>
     <row r="180" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B180" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F180"/>
       <c r="G180" s="10"/>
@@ -4481,21 +4484,21 @@
       </c>
       <c r="I180" s="10"/>
       <c r="K180" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M180" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="O180" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="Q180" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="181" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C181">
         <v>2</v>
@@ -4511,14 +4514,14 @@
       </c>
       <c r="K181"/>
       <c r="L181" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="O181"/>
       <c r="Q181"/>
     </row>
     <row r="182" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B182" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F182"/>
       <c r="G182" s="10"/>
@@ -4527,14 +4530,14 @@
         <v>14</v>
       </c>
       <c r="M182" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="O182"/>
       <c r="Q182"/>
     </row>
     <row r="183" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C183" s="10">
         <v>3</v>
@@ -4557,7 +4560,7 @@
     </row>
     <row r="184" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B184" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F184"/>
       <c r="G184" s="10"/>
@@ -4598,7 +4601,7 @@
     </row>
     <row r="188" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A188" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="189" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -4654,7 +4657,7 @@
     </row>
     <row r="191" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C191" s="10">
         <v>1</v>
@@ -4675,7 +4678,7 @@
     </row>
     <row r="192" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B192" s="4" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C192" s="10"/>
       <c r="D192" s="10"/>
@@ -4690,7 +4693,7 @@
     </row>
     <row r="193" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C193" s="10">
         <v>4</v>
@@ -4709,7 +4712,7 @@
     </row>
     <row r="194" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B194" s="4" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C194" s="10"/>
       <c r="D194" s="10"/>
@@ -4717,7 +4720,7 @@
       <c r="F194"/>
       <c r="J194" s="10"/>
       <c r="K194" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="M194"/>
       <c r="O194"/>
@@ -4725,7 +4728,7 @@
     </row>
     <row r="195" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C195" s="10">
         <v>2</v>
@@ -4739,7 +4742,7 @@
       <c r="H195"/>
       <c r="K195"/>
       <c r="L195" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="M195"/>
       <c r="N195">
@@ -4753,7 +4756,7 @@
     </row>
     <row r="196" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B196" s="4" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C196" s="10"/>
       <c r="D196" s="10"/>
@@ -4763,18 +4766,18 @@
       <c r="H196"/>
       <c r="K196"/>
       <c r="M196" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="O196" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="Q196" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="197" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C197" s="10">
         <v>3</v>
@@ -4790,7 +4793,7 @@
         <v>0.12</v>
       </c>
       <c r="L197" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N197">
         <v>6</v>
@@ -4803,7 +4806,7 @@
     </row>
     <row r="198" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B198" s="4" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C198" s="10"/>
       <c r="D198" s="10"/>
@@ -4811,21 +4814,21 @@
         <v>58</v>
       </c>
       <c r="K198" t="s">
+        <v>198</v>
+      </c>
+      <c r="M198" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="O198" t="s">
         <v>200</v>
       </c>
-      <c r="M198" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="O198" t="s">
-        <v>202</v>
-      </c>
       <c r="Q198" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="199" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C199" s="10">
         <v>1</v>
@@ -4846,7 +4849,7 @@
     </row>
     <row r="200" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B200" s="4" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C200" s="10"/>
       <c r="D200" s="10"/>
@@ -4861,7 +4864,7 @@
     </row>
     <row r="201" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C201" s="10"/>
       <c r="D201" s="10">
@@ -4884,7 +4887,7 @@
     </row>
     <row r="202" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B202" s="4" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C202" s="10"/>
       <c r="D202" s="10"/>
@@ -4932,21 +4935,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d42a73f51a03135be35f4acb272f8cf1">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ea21b36c10eaa86a5cb337ec7f4e0a6" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3dd70bd28c77d4108edb5ca6812bb84f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cd59d6f2988212fc297a6d404d3fed4" ns2:_="" ns3:_="">
     <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
     <xsd:import namespace="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
     <xsd:element name="properties">
@@ -5199,6 +5194,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5211,6 +5215,10 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{256A220B-D155-4F0E-9C02-F717E97A8446}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB7E9D24-58F4-4B3F-86E2-7E155CA9AA5C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -5218,23 +5226,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75A78422-BADC-4FBE-8DA4-B601C8891818}"/>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15DF461F-679A-46D8-ABBB-E1327B97C2C5}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>